<commit_message>
Add E2E tests for CRUD operations on pets, including validation for duplicate IDs and negative weights
</commit_message>
<xml_diff>
--- a/cypress/testdata/Dataset-Escenarios-PETS-SA.xlsx
+++ b/cypress/testdata/Dataset-Escenarios-PETS-SA.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bolis\Downloads\Gestión de pruebas\pets-sa-suite-java\src\test\resources\dataset\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bolis\Downloads\Gestión de pruebas\cypress-pets-sa\cypress\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3FCE3E5-EE94-446D-870D-6B4DD578476F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7E35505-971C-441B-A1F9-B9D68D91816B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="11295" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ESC01_XSS_SQLI" sheetId="8" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="471" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="185">
   <si>
     <t>CLI</t>
   </si>
@@ -561,6 +561,24 @@
   </si>
   <si>
     <t>MASC-002</t>
+  </si>
+  <si>
+    <t>M-I-02</t>
+  </si>
+  <si>
+    <t>-5.00</t>
+  </si>
+  <si>
+    <t>Peso negativo no debe aceptarse</t>
+  </si>
+  <si>
+    <t>MASC-004</t>
+  </si>
+  <si>
+    <t>Rocky</t>
+  </si>
+  <si>
+    <t>Husky</t>
   </si>
 </sst>
 </file>
@@ -1062,180 +1080,180 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CE2DFEBB-5EDB-44B1-8874-57648884DCDB}" name="Tabla1" displayName="Tabla1" ref="A1:AB3" totalsRowShown="0" headerRowDxfId="109" dataDxfId="108">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CE2DFEBB-5EDB-44B1-8874-57648884DCDB}" name="Tabla1" displayName="Tabla1" ref="A1:AB3" totalsRowShown="0" headerRowDxfId="111" dataDxfId="110">
   <autoFilter ref="A1:AB3" xr:uid="{CE2DFEBB-5EDB-44B1-8874-57648884DCDB}"/>
   <tableColumns count="28">
-    <tableColumn id="28" xr3:uid="{91572F6C-9293-44C1-8F7E-EF820C3FC134}" name="* Test Cases*" dataDxfId="107"/>
-    <tableColumn id="1" xr3:uid="{A9A7F625-F933-44B0-86A1-01175AC9D71B}" name="${module}" dataDxfId="106"/>
-    <tableColumn id="2" xr3:uid="{E5F7A95A-DBBB-4162-9672-82DC7BAD6E66}" name="${dataset_id}" dataDxfId="105"/>
-    <tableColumn id="3" xr3:uid="{48951BA2-790A-4CDA-9C8E-403D02FD7C3F}" name="${modulo}" dataDxfId="104"/>
-    <tableColumn id="4" xr3:uid="{9D53264E-B20A-49F1-8EF2-52DC154C0647}" name="${cedula}" dataDxfId="103"/>
-    <tableColumn id="5" xr3:uid="{9B96DF8B-9E57-432D-9405-AC795A232AFE}" name="${nombres}" dataDxfId="102"/>
-    <tableColumn id="6" xr3:uid="{00609FF2-0D99-4D65-B2E2-59765A4CD032}" name="${apellidos}" dataDxfId="101"/>
-    <tableColumn id="7" xr3:uid="{7EA18710-98C2-40A2-96BA-1BEDCF391884}" name="${telefono}" dataDxfId="100"/>
-    <tableColumn id="8" xr3:uid="{4777E89D-0047-4406-9581-CF86AAD87F97}" name="${direccion}" dataDxfId="99"/>
-    <tableColumn id="9" xr3:uid="{89132D6D-7B87-4DDB-B160-74769410B37A}" name="${med_nombre}" dataDxfId="98"/>
-    <tableColumn id="10" xr3:uid="{5F77B49C-2B90-4290-BF4E-27354B0CCB96}" name="${med_descripcion}" dataDxfId="97"/>
-    <tableColumn id="11" xr3:uid="{2F36F9D9-9B7E-46D2-881B-E79ACD6A83F0}" name="${med_dosis}" dataDxfId="96"/>
-    <tableColumn id="12" xr3:uid="{4E7E7AD7-1E1D-4A34-9C35-20D6DB4C3573}" name="${tipo}" dataDxfId="95"/>
-    <tableColumn id="13" xr3:uid="{EFC25A82-DB7A-4B87-B147-5248BF3C87FF}" name="${expected_result}" dataDxfId="94"/>
-    <tableColumn id="14" xr3:uid="{BD5932A9-A5EE-4E1B-8ED6-6A103B3DDC2A}" name="${RF}" dataDxfId="93"/>
-    <tableColumn id="15" xr3:uid="{9B57296F-1147-4A3C-8DA3-124069878685}" name="${accion}" dataDxfId="92"/>
-    <tableColumn id="16" xr3:uid="{8C4E9941-9A6D-4655-897B-D4596C15B48C}" name="${nota_defecto}" dataDxfId="91"/>
-    <tableColumn id="17" xr3:uid="{0AE6C3EB-FC04-4E96-8012-20B136D1C8F8}" name="${estado_bug}" dataDxfId="90"/>
-    <tableColumn id="18" xr3:uid="{A4C2532E-C6D5-482F-9745-D650E08635C5}" name="${campo_f1_locator}" dataDxfId="89"/>
-    <tableColumn id="19" xr3:uid="{B0D6C91C-9E3D-41B8-9352-AEB2E5117F17}" name="${campo_f2_locator}" dataDxfId="88"/>
-    <tableColumn id="20" xr3:uid="{3AC77FD5-E18A-41F7-9209-715EAAFD94A0}" name="${campo_f3_locator}" dataDxfId="87"/>
-    <tableColumn id="21" xr3:uid="{1B17F57F-3951-423C-B181-4F2C7AD4A8D9}" name="${campo_f4_locator}" dataDxfId="86"/>
-    <tableColumn id="22" xr3:uid="{B97B8F3A-C4B9-432C-B0FD-35A18C9FB431}" name="${campo_f5_locator}" dataDxfId="85"/>
-    <tableColumn id="23" xr3:uid="{699D4D33-9D9B-4CCD-920B-ECB9D7F5A5C3}" name="${campo_submit_locator}" dataDxfId="84"/>
-    <tableColumn id="24" xr3:uid="{24699C7C-0B93-429C-9F2B-6A68326D2206}" name="${campo_listado_locator}" dataDxfId="83"/>
-    <tableColumn id="25" xr3:uid="{C80F56F2-5F93-4BC3-B99F-FBD433939027}" name="${campo_error_locator}" dataDxfId="82"/>
-    <tableColumn id="26" xr3:uid="{5FC366F9-C83D-46FE-BC66-331C097465C9}" name="${username}" dataDxfId="81"/>
-    <tableColumn id="27" xr3:uid="{2F2F6D69-B858-4D80-916D-844FD07B853B}" name="${password}" dataDxfId="80"/>
+    <tableColumn id="28" xr3:uid="{91572F6C-9293-44C1-8F7E-EF820C3FC134}" name="* Test Cases*" dataDxfId="109"/>
+    <tableColumn id="1" xr3:uid="{A9A7F625-F933-44B0-86A1-01175AC9D71B}" name="${module}" dataDxfId="108"/>
+    <tableColumn id="2" xr3:uid="{E5F7A95A-DBBB-4162-9672-82DC7BAD6E66}" name="${dataset_id}" dataDxfId="107"/>
+    <tableColumn id="3" xr3:uid="{48951BA2-790A-4CDA-9C8E-403D02FD7C3F}" name="${modulo}" dataDxfId="106"/>
+    <tableColumn id="4" xr3:uid="{9D53264E-B20A-49F1-8EF2-52DC154C0647}" name="${cedula}" dataDxfId="105"/>
+    <tableColumn id="5" xr3:uid="{9B96DF8B-9E57-432D-9405-AC795A232AFE}" name="${nombres}" dataDxfId="104"/>
+    <tableColumn id="6" xr3:uid="{00609FF2-0D99-4D65-B2E2-59765A4CD032}" name="${apellidos}" dataDxfId="103"/>
+    <tableColumn id="7" xr3:uid="{7EA18710-98C2-40A2-96BA-1BEDCF391884}" name="${telefono}" dataDxfId="102"/>
+    <tableColumn id="8" xr3:uid="{4777E89D-0047-4406-9581-CF86AAD87F97}" name="${direccion}" dataDxfId="101"/>
+    <tableColumn id="9" xr3:uid="{89132D6D-7B87-4DDB-B160-74769410B37A}" name="${med_nombre}" dataDxfId="100"/>
+    <tableColumn id="10" xr3:uid="{5F77B49C-2B90-4290-BF4E-27354B0CCB96}" name="${med_descripcion}" dataDxfId="99"/>
+    <tableColumn id="11" xr3:uid="{2F36F9D9-9B7E-46D2-881B-E79ACD6A83F0}" name="${med_dosis}" dataDxfId="98"/>
+    <tableColumn id="12" xr3:uid="{4E7E7AD7-1E1D-4A34-9C35-20D6DB4C3573}" name="${tipo}" dataDxfId="97"/>
+    <tableColumn id="13" xr3:uid="{EFC25A82-DB7A-4B87-B147-5248BF3C87FF}" name="${expected_result}" dataDxfId="96"/>
+    <tableColumn id="14" xr3:uid="{BD5932A9-A5EE-4E1B-8ED6-6A103B3DDC2A}" name="${RF}" dataDxfId="95"/>
+    <tableColumn id="15" xr3:uid="{9B57296F-1147-4A3C-8DA3-124069878685}" name="${accion}" dataDxfId="94"/>
+    <tableColumn id="16" xr3:uid="{8C4E9941-9A6D-4655-897B-D4596C15B48C}" name="${nota_defecto}" dataDxfId="93"/>
+    <tableColumn id="17" xr3:uid="{0AE6C3EB-FC04-4E96-8012-20B136D1C8F8}" name="${estado_bug}" dataDxfId="92"/>
+    <tableColumn id="18" xr3:uid="{A4C2532E-C6D5-482F-9745-D650E08635C5}" name="${campo_f1_locator}" dataDxfId="91"/>
+    <tableColumn id="19" xr3:uid="{B0D6C91C-9E3D-41B8-9352-AEB2E5117F17}" name="${campo_f2_locator}" dataDxfId="90"/>
+    <tableColumn id="20" xr3:uid="{3AC77FD5-E18A-41F7-9209-715EAAFD94A0}" name="${campo_f3_locator}" dataDxfId="89"/>
+    <tableColumn id="21" xr3:uid="{1B17F57F-3951-423C-B181-4F2C7AD4A8D9}" name="${campo_f4_locator}" dataDxfId="88"/>
+    <tableColumn id="22" xr3:uid="{B97B8F3A-C4B9-432C-B0FD-35A18C9FB431}" name="${campo_f5_locator}" dataDxfId="87"/>
+    <tableColumn id="23" xr3:uid="{699D4D33-9D9B-4CCD-920B-ECB9D7F5A5C3}" name="${campo_submit_locator}" dataDxfId="86"/>
+    <tableColumn id="24" xr3:uid="{24699C7C-0B93-429C-9F2B-6A68326D2206}" name="${campo_listado_locator}" dataDxfId="85"/>
+    <tableColumn id="25" xr3:uid="{C80F56F2-5F93-4BC3-B99F-FBD433939027}" name="${campo_error_locator}" dataDxfId="84"/>
+    <tableColumn id="26" xr3:uid="{5FC366F9-C83D-46FE-BC66-331C097465C9}" name="${username}" dataDxfId="83"/>
+    <tableColumn id="27" xr3:uid="{2F2F6D69-B858-4D80-916D-844FD07B853B}" name="${password}" dataDxfId="82"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{883D2E49-F209-4069-A921-67DD725DF7A9}" name="Tabla2" displayName="Tabla2" ref="A1:U5" totalsRowShown="0" headerRowDxfId="79" dataDxfId="78">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{883D2E49-F209-4069-A921-67DD725DF7A9}" name="Tabla2" displayName="Tabla2" ref="A1:U5" totalsRowShown="0" headerRowDxfId="81" dataDxfId="80">
   <autoFilter ref="A1:U5" xr:uid="{883D2E49-F209-4069-A921-67DD725DF7A9}"/>
   <tableColumns count="21">
-    <tableColumn id="21" xr3:uid="{00D3C5F7-6059-4A65-8FED-E0B14D83839F}" name="* Test Cases*" dataDxfId="77"/>
-    <tableColumn id="1" xr3:uid="{97231F21-6B84-40A6-9AAA-1FD6F7049CBC}" name="${module}" dataDxfId="76"/>
-    <tableColumn id="2" xr3:uid="{97562332-401B-4700-B619-39D147FC073C}" name="${dataset_id}" dataDxfId="75"/>
-    <tableColumn id="3" xr3:uid="{DF36D72A-34C7-44E4-866B-2CB0DD6A9B0A}" name="${username}" dataDxfId="74"/>
-    <tableColumn id="4" xr3:uid="{813BFD25-6670-4A22-832A-F88F16F607DF}" name="${password}" dataDxfId="73"/>
-    <tableColumn id="5" xr3:uid="{283E7CAE-4A63-41F8-B803-46F502A84992}" name="${role}" dataDxfId="72"/>
-    <tableColumn id="6" xr3:uid="{B228DF6D-141F-434A-9DBC-8AE456714A4E}" name="${tipo}" dataDxfId="71"/>
-    <tableColumn id="7" xr3:uid="{204905D5-1606-45A5-985D-2F7AC7BDD09B}" name="${expected_result}" dataDxfId="70"/>
-    <tableColumn id="8" xr3:uid="{D080A1AC-8029-461B-9AB5-30D629C85B04}" name="${RF}" dataDxfId="69"/>
-    <tableColumn id="9" xr3:uid="{99586779-32EC-4991-8921-D9FDCFAC827C}" name="${accion}" dataDxfId="68"/>
-    <tableColumn id="10" xr3:uid="{1C402D8C-3783-4458-BC41-8A849DE179DE}" name="${campo_url_login}" dataDxfId="67"/>
-    <tableColumn id="11" xr3:uid="{1E1F04B6-F134-4B62-A058-88E5DDEC4E74}" name="${campo_url_target}" dataDxfId="66"/>
-    <tableColumn id="12" xr3:uid="{70136979-209D-44B6-ACBD-DF9A0C7FB1EA}" name="${campo_url_denied}" dataDxfId="65"/>
-    <tableColumn id="13" xr3:uid="{A5036F18-29E2-4811-9B1C-FC03BD796786}" name="${campo_user_locator}" dataDxfId="64"/>
-    <tableColumn id="14" xr3:uid="{3BF94819-B4EE-4D05-B827-C1BD5E12CEBC}" name="${campo_pass_locator}" dataDxfId="63"/>
-    <tableColumn id="15" xr3:uid="{C996B767-EEC3-4617-81E1-5E8B3B6B776C}" name="${campo_submit_locator}" dataDxfId="62"/>
-    <tableColumn id="16" xr3:uid="{9384D189-B91A-4444-AC0F-EA9578057215}" name="${campo_dashboard_locator}" dataDxfId="61"/>
-    <tableColumn id="17" xr3:uid="{504D1857-FB02-45D9-B073-6AD40FF0DC34}" name="${campo_logout_locator}" dataDxfId="60"/>
-    <tableColumn id="18" xr3:uid="{2462D9E6-F8BD-44AD-895E-F76171E4BCD1}" name="${campo_error_locator}" dataDxfId="59"/>
-    <tableColumn id="19" xr3:uid="{D10626BC-A516-4CC7-9AFE-18819824E3DB}" name="${expected_error_text}" dataDxfId="58"/>
-    <tableColumn id="20" xr3:uid="{78A604AA-4A4A-4105-92F8-158BA9A9DD95}" name="${estado_bug}" dataDxfId="57"/>
+    <tableColumn id="21" xr3:uid="{00D3C5F7-6059-4A65-8FED-E0B14D83839F}" name="* Test Cases*" dataDxfId="79"/>
+    <tableColumn id="1" xr3:uid="{97231F21-6B84-40A6-9AAA-1FD6F7049CBC}" name="${module}" dataDxfId="78"/>
+    <tableColumn id="2" xr3:uid="{97562332-401B-4700-B619-39D147FC073C}" name="${dataset_id}" dataDxfId="77"/>
+    <tableColumn id="3" xr3:uid="{DF36D72A-34C7-44E4-866B-2CB0DD6A9B0A}" name="${username}" dataDxfId="76"/>
+    <tableColumn id="4" xr3:uid="{813BFD25-6670-4A22-832A-F88F16F607DF}" name="${password}" dataDxfId="75"/>
+    <tableColumn id="5" xr3:uid="{283E7CAE-4A63-41F8-B803-46F502A84992}" name="${role}" dataDxfId="74"/>
+    <tableColumn id="6" xr3:uid="{B228DF6D-141F-434A-9DBC-8AE456714A4E}" name="${tipo}" dataDxfId="73"/>
+    <tableColumn id="7" xr3:uid="{204905D5-1606-45A5-985D-2F7AC7BDD09B}" name="${expected_result}" dataDxfId="72"/>
+    <tableColumn id="8" xr3:uid="{D080A1AC-8029-461B-9AB5-30D629C85B04}" name="${RF}" dataDxfId="71"/>
+    <tableColumn id="9" xr3:uid="{99586779-32EC-4991-8921-D9FDCFAC827C}" name="${accion}" dataDxfId="70"/>
+    <tableColumn id="10" xr3:uid="{1C402D8C-3783-4458-BC41-8A849DE179DE}" name="${campo_url_login}" dataDxfId="69"/>
+    <tableColumn id="11" xr3:uid="{1E1F04B6-F134-4B62-A058-88E5DDEC4E74}" name="${campo_url_target}" dataDxfId="68"/>
+    <tableColumn id="12" xr3:uid="{70136979-209D-44B6-ACBD-DF9A0C7FB1EA}" name="${campo_url_denied}" dataDxfId="67"/>
+    <tableColumn id="13" xr3:uid="{A5036F18-29E2-4811-9B1C-FC03BD796786}" name="${campo_user_locator}" dataDxfId="66"/>
+    <tableColumn id="14" xr3:uid="{3BF94819-B4EE-4D05-B827-C1BD5E12CEBC}" name="${campo_pass_locator}" dataDxfId="65"/>
+    <tableColumn id="15" xr3:uid="{C996B767-EEC3-4617-81E1-5E8B3B6B776C}" name="${campo_submit_locator}" dataDxfId="64"/>
+    <tableColumn id="16" xr3:uid="{9384D189-B91A-4444-AC0F-EA9578057215}" name="${campo_dashboard_locator}" dataDxfId="63"/>
+    <tableColumn id="17" xr3:uid="{504D1857-FB02-45D9-B073-6AD40FF0DC34}" name="${campo_logout_locator}" dataDxfId="62"/>
+    <tableColumn id="18" xr3:uid="{2462D9E6-F8BD-44AD-895E-F76171E4BCD1}" name="${campo_error_locator}" dataDxfId="61"/>
+    <tableColumn id="19" xr3:uid="{D10626BC-A516-4CC7-9AFE-18819824E3DB}" name="${expected_error_text}" dataDxfId="60"/>
+    <tableColumn id="20" xr3:uid="{78A604AA-4A4A-4105-92F8-158BA9A9DD95}" name="${estado_bug}" dataDxfId="59"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{FEB12AEE-7D6C-454A-A24C-9AA9E2B99069}" name="Tabla8" displayName="Tabla8" ref="A1:AG3" totalsRowShown="0" headerRowDxfId="144" dataDxfId="143">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{FEB12AEE-7D6C-454A-A24C-9AA9E2B99069}" name="Tabla8" displayName="Tabla8" ref="A1:AG3" totalsRowShown="0" headerRowDxfId="58" dataDxfId="57">
   <autoFilter ref="A1:AG3" xr:uid="{FEB12AEE-7D6C-454A-A24C-9AA9E2B99069}"/>
   <tableColumns count="33">
-    <tableColumn id="33" xr3:uid="{A3A7A5FE-1241-482B-A5C1-E69AD1216F8D}" name="* Test Cases*" dataDxfId="142"/>
-    <tableColumn id="2" xr3:uid="{031EBE7C-5E22-485D-B14E-F8F3CF9E30BB}" name="${module}" dataDxfId="141"/>
-    <tableColumn id="3" xr3:uid="{64102414-FFB9-4405-B0E9-9F48A580ED20}" name="${dataset_id}" dataDxfId="140"/>
-    <tableColumn id="4" xr3:uid="{A22418AA-E9E2-4833-BFFD-EAD04067B76D}" name="${modulo}" dataDxfId="139"/>
-    <tableColumn id="5" xr3:uid="{74A259D3-8C4A-455F-BE65-600402C6A754}" name="${username}" dataDxfId="138"/>
-    <tableColumn id="6" xr3:uid="{46BC6221-10EB-4C01-A4A8-6DCF6BD753E6}" name="${password}" dataDxfId="137"/>
-    <tableColumn id="7" xr3:uid="{1A696440-5CAD-4450-A245-A132D9303E8C}" name="${cedula}" dataDxfId="136"/>
-    <tableColumn id="8" xr3:uid="{1F8B8908-8064-43B4-A0DA-327299FEAFD5}" name="${nombres}" dataDxfId="135"/>
-    <tableColumn id="9" xr3:uid="{8055B264-C604-4D60-BAD6-F648B0BA66BD}" name="${apellidos}" dataDxfId="134"/>
-    <tableColumn id="10" xr3:uid="{ACAFA784-697B-42ED-A9F6-ECB17C5E8651}" name="${telefono}" dataDxfId="133"/>
-    <tableColumn id="11" xr3:uid="{AB21A3C2-9379-4762-8EEB-231CC043BA9E}" name="${direccion}" dataDxfId="132"/>
-    <tableColumn id="12" xr3:uid="{AE4269B5-AD3F-4371-B1AF-1F96FC572DB7}" name="${pet_id}" dataDxfId="131"/>
-    <tableColumn id="13" xr3:uid="{282F5CEB-9C74-42A1-A790-592689B20839}" name="${nombre_mascota}" dataDxfId="130"/>
-    <tableColumn id="14" xr3:uid="{D808A2E7-0843-4905-80B4-3E9B246C95DC}" name="${raza}" dataDxfId="129"/>
-    <tableColumn id="15" xr3:uid="{813D1117-EF28-4D37-8006-C14E461ED0E7}" name="${edad}" dataDxfId="128"/>
-    <tableColumn id="16" xr3:uid="{357997B2-5834-46D4-A46E-F90494036763}" name="${peso}" dataDxfId="127"/>
-    <tableColumn id="17" xr3:uid="{8DE2879D-ABBB-4C52-B15B-0B2A2D459325}" name="${cliente_id}" dataDxfId="126"/>
-    <tableColumn id="18" xr3:uid="{54C6811B-04B4-4165-8750-1378D9484C9C}" name="${tipo}" dataDxfId="125"/>
-    <tableColumn id="19" xr3:uid="{1A22608F-BCE8-44AB-A78A-B8931D0B43B2}" name="${expected_result}" dataDxfId="124"/>
-    <tableColumn id="20" xr3:uid="{10DF7064-FEB5-4737-A0DC-9DF2338B0C97}" name="${RF}" dataDxfId="123"/>
-    <tableColumn id="21" xr3:uid="{FEC51B1A-F3D1-4717-9FE3-6D9163FB2A31}" name="${accion}" dataDxfId="122"/>
-    <tableColumn id="22" xr3:uid="{026C4213-221E-41DC-98B7-5A1CE5E5F0C9}" name="${nota_defecto}" dataDxfId="121"/>
-    <tableColumn id="23" xr3:uid="{CD67DA82-3E02-44BA-A5E1-29ADE4459B0F}" name="${estado_bug}" dataDxfId="120"/>
-    <tableColumn id="24" xr3:uid="{6C97B18F-B7D8-4A6C-A6FA-A111CC0D14AB}" name="${campo_f1_locator}" dataDxfId="119"/>
-    <tableColumn id="25" xr3:uid="{62A8B345-CC27-41AB-807A-2F6D46F7DCE1}" name="${campo_f2_locator}" dataDxfId="118"/>
-    <tableColumn id="26" xr3:uid="{DDAFE9A5-BC27-4C04-9227-CA3AA80AAD28}" name="${campo_f3_locator}" dataDxfId="117"/>
-    <tableColumn id="27" xr3:uid="{9BB95DF5-4BBC-44EB-AD25-BF92D23E6396}" name="${campo_f4_locator}" dataDxfId="116"/>
-    <tableColumn id="28" xr3:uid="{EA17C1DD-F10F-41F7-8F11-C03C5B29395C}" name="${campo_f5_locator}" dataDxfId="115"/>
-    <tableColumn id="29" xr3:uid="{965DC346-0DFD-44A5-9819-164292565F7E}" name="${campo_cliente_locator}" dataDxfId="114"/>
-    <tableColumn id="30" xr3:uid="{076F0B0E-8E04-4A64-BF67-62F6668FB176}" name="${campo_submit_locator}" dataDxfId="113"/>
-    <tableColumn id="1" xr3:uid="{4E75182C-453E-4F12-8896-8C02A558828C}" name="${campo_listado_locator}" dataDxfId="112"/>
-    <tableColumn id="31" xr3:uid="{9193C99C-D877-4073-8762-7A27F2629728}" name="${campo_error_locator}" dataDxfId="111"/>
-    <tableColumn id="32" xr3:uid="{C25C84A8-BFC7-4AB8-91CA-3B171BF6246B}" name="${expected_error_text}" dataDxfId="110"/>
+    <tableColumn id="33" xr3:uid="{A3A7A5FE-1241-482B-A5C1-E69AD1216F8D}" name="* Test Cases*" dataDxfId="56"/>
+    <tableColumn id="2" xr3:uid="{031EBE7C-5E22-485D-B14E-F8F3CF9E30BB}" name="${module}" dataDxfId="55"/>
+    <tableColumn id="3" xr3:uid="{64102414-FFB9-4405-B0E9-9F48A580ED20}" name="${dataset_id}" dataDxfId="54"/>
+    <tableColumn id="4" xr3:uid="{A22418AA-E9E2-4833-BFFD-EAD04067B76D}" name="${modulo}" dataDxfId="53"/>
+    <tableColumn id="5" xr3:uid="{74A259D3-8C4A-455F-BE65-600402C6A754}" name="${username}" dataDxfId="52"/>
+    <tableColumn id="6" xr3:uid="{46BC6221-10EB-4C01-A4A8-6DCF6BD753E6}" name="${password}" dataDxfId="51"/>
+    <tableColumn id="7" xr3:uid="{1A696440-5CAD-4450-A245-A132D9303E8C}" name="${cedula}" dataDxfId="50"/>
+    <tableColumn id="8" xr3:uid="{1F8B8908-8064-43B4-A0DA-327299FEAFD5}" name="${nombres}" dataDxfId="49"/>
+    <tableColumn id="9" xr3:uid="{8055B264-C604-4D60-BAD6-F648B0BA66BD}" name="${apellidos}" dataDxfId="48"/>
+    <tableColumn id="10" xr3:uid="{ACAFA784-697B-42ED-A9F6-ECB17C5E8651}" name="${telefono}" dataDxfId="47"/>
+    <tableColumn id="11" xr3:uid="{AB21A3C2-9379-4762-8EEB-231CC043BA9E}" name="${direccion}" dataDxfId="46"/>
+    <tableColumn id="12" xr3:uid="{AE4269B5-AD3F-4371-B1AF-1F96FC572DB7}" name="${pet_id}" dataDxfId="45"/>
+    <tableColumn id="13" xr3:uid="{282F5CEB-9C74-42A1-A790-592689B20839}" name="${nombre_mascota}" dataDxfId="44"/>
+    <tableColumn id="14" xr3:uid="{D808A2E7-0843-4905-80B4-3E9B246C95DC}" name="${raza}" dataDxfId="43"/>
+    <tableColumn id="15" xr3:uid="{813D1117-EF28-4D37-8006-C14E461ED0E7}" name="${edad}" dataDxfId="42"/>
+    <tableColumn id="16" xr3:uid="{357997B2-5834-46D4-A46E-F90494036763}" name="${peso}" dataDxfId="41"/>
+    <tableColumn id="17" xr3:uid="{8DE2879D-ABBB-4C52-B15B-0B2A2D459325}" name="${cliente_id}" dataDxfId="40"/>
+    <tableColumn id="18" xr3:uid="{54C6811B-04B4-4165-8750-1378D9484C9C}" name="${tipo}" dataDxfId="39"/>
+    <tableColumn id="19" xr3:uid="{1A22608F-BCE8-44AB-A78A-B8931D0B43B2}" name="${expected_result}" dataDxfId="38"/>
+    <tableColumn id="20" xr3:uid="{10DF7064-FEB5-4737-A0DC-9DF2338B0C97}" name="${RF}" dataDxfId="37"/>
+    <tableColumn id="21" xr3:uid="{FEC51B1A-F3D1-4717-9FE3-6D9163FB2A31}" name="${accion}" dataDxfId="36"/>
+    <tableColumn id="22" xr3:uid="{026C4213-221E-41DC-98B7-5A1CE5E5F0C9}" name="${nota_defecto}" dataDxfId="35"/>
+    <tableColumn id="23" xr3:uid="{CD67DA82-3E02-44BA-A5E1-29ADE4459B0F}" name="${estado_bug}" dataDxfId="34"/>
+    <tableColumn id="24" xr3:uid="{6C97B18F-B7D8-4A6C-A6FA-A111CC0D14AB}" name="${campo_f1_locator}" dataDxfId="33"/>
+    <tableColumn id="25" xr3:uid="{62A8B345-CC27-41AB-807A-2F6D46F7DCE1}" name="${campo_f2_locator}" dataDxfId="32"/>
+    <tableColumn id="26" xr3:uid="{DDAFE9A5-BC27-4C04-9227-CA3AA80AAD28}" name="${campo_f3_locator}" dataDxfId="31"/>
+    <tableColumn id="27" xr3:uid="{9BB95DF5-4BBC-44EB-AD25-BF92D23E6396}" name="${campo_f4_locator}" dataDxfId="30"/>
+    <tableColumn id="28" xr3:uid="{EA17C1DD-F10F-41F7-8F11-C03C5B29395C}" name="${campo_f5_locator}" dataDxfId="29"/>
+    <tableColumn id="29" xr3:uid="{965DC346-0DFD-44A5-9819-164292565F7E}" name="${campo_cliente_locator}" dataDxfId="28"/>
+    <tableColumn id="30" xr3:uid="{076F0B0E-8E04-4A64-BF67-62F6668FB176}" name="${campo_submit_locator}" dataDxfId="27"/>
+    <tableColumn id="1" xr3:uid="{4E75182C-453E-4F12-8896-8C02A558828C}" name="${campo_listado_locator}" dataDxfId="26"/>
+    <tableColumn id="31" xr3:uid="{9193C99C-D877-4073-8762-7A27F2629728}" name="${campo_error_locator}" dataDxfId="25"/>
+    <tableColumn id="32" xr3:uid="{C25C84A8-BFC7-4AB8-91CA-3B171BF6246B}" name="${expected_error_text}" dataDxfId="24"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{4060F21C-5DF4-4C48-A2E8-B4B9442A1BC9}" name="Tabla5" displayName="Tabla5" ref="A1:V5" totalsRowShown="0" headerRowDxfId="56" dataDxfId="55">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{4060F21C-5DF4-4C48-A2E8-B4B9442A1BC9}" name="Tabla5" displayName="Tabla5" ref="A1:V5" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
   <autoFilter ref="A1:V5" xr:uid="{4060F21C-5DF4-4C48-A2E8-B4B9442A1BC9}"/>
   <tableColumns count="22">
-    <tableColumn id="22" xr3:uid="{C8403B0F-0195-4D46-A1A3-D24E124BE6E5}" name="* Test Cases*" dataDxfId="54"/>
-    <tableColumn id="1" xr3:uid="{4976F6FD-69E7-46E4-B49F-470CB1054B48}" name="${module}" dataDxfId="53"/>
-    <tableColumn id="2" xr3:uid="{F5245C18-BA71-4C91-88F9-FA238A6A2D4D}" name="${dataset_id}" dataDxfId="52"/>
-    <tableColumn id="3" xr3:uid="{4046FD08-D747-4231-82F5-17A600D3E724}" name="${username}" dataDxfId="51"/>
-    <tableColumn id="4" xr3:uid="{FBEEF32A-E8E8-4E6F-A05E-10E6A4689538}" name="${password}" dataDxfId="50"/>
-    <tableColumn id="5" xr3:uid="{BBBF3383-D2A3-443A-B066-35CEBE6A0DCF}" name="${role}" dataDxfId="49"/>
-    <tableColumn id="6" xr3:uid="{FFF3448B-D728-4BFB-8F56-81A8FC0AC0DC}" name="${tipo}" dataDxfId="48"/>
-    <tableColumn id="7" xr3:uid="{627C75CC-31B9-4230-8E9A-6B2A4F1A3E6F}" name="${expected_result}" dataDxfId="47"/>
-    <tableColumn id="8" xr3:uid="{DA869EDF-F801-447F-AB76-1E28982A4E9D}" name="${RF}" dataDxfId="46"/>
-    <tableColumn id="9" xr3:uid="{40726AA5-C158-4170-AF35-03DBF46E59E6}" name="${accion}" dataDxfId="45"/>
-    <tableColumn id="10" xr3:uid="{F473F2A5-D7E5-40FF-80EF-B18B0504175C}" name="${campo_url_login}" dataDxfId="44"/>
-    <tableColumn id="11" xr3:uid="{E4A9ED2B-154A-4E07-A3D3-3E8B0EB7662A}" name="${campo_url_target}" dataDxfId="43"/>
-    <tableColumn id="12" xr3:uid="{74E8A3EF-3F1F-4E69-82DE-3C0D9FF3BFF1}" name="${campo_user_locator}" dataDxfId="42"/>
-    <tableColumn id="13" xr3:uid="{FDE67EA9-2B9C-46D5-9C05-283FC050BB68}" name="${campo_pass_locator}" dataDxfId="41"/>
-    <tableColumn id="14" xr3:uid="{3F4A6565-B175-4200-8CD1-D2AA0122ABD9}" name="${campo_submit_locator}" dataDxfId="40"/>
-    <tableColumn id="15" xr3:uid="{2AF443CA-A5EA-401B-9777-981D622C02EF}" name="${campo_dashboard_locator}" dataDxfId="39"/>
-    <tableColumn id="16" xr3:uid="{83424C47-D770-4BE9-8442-5725F667ECD1}" name="${campo_logout_locator}" dataDxfId="38"/>
-    <tableColumn id="17" xr3:uid="{7EEE2949-909D-410F-952D-B9F1D152C5AD}" name="${campo_error_locator}" dataDxfId="37"/>
-    <tableColumn id="18" xr3:uid="{1F68B334-E4E9-4EEE-A3E4-188E3AFD24EA}" name="${expected_error_text}" dataDxfId="36"/>
-    <tableColumn id="19" xr3:uid="{6956A1B5-B972-4BEB-80EF-AE0E78A64242}" name="${campo_bloqueo_locator}" dataDxfId="35"/>
-    <tableColumn id="20" xr3:uid="{F4C1388D-5BD9-4F61-8FCF-C13B6D0FB785}" name="${expected_bloqueo_text}" dataDxfId="34"/>
-    <tableColumn id="21" xr3:uid="{6B400DAD-0A5C-45C1-AE39-96C60BBDC24C}" name="${estado_bug}" dataDxfId="33"/>
+    <tableColumn id="22" xr3:uid="{C8403B0F-0195-4D46-A1A3-D24E124BE6E5}" name="* Test Cases*" dataDxfId="21"/>
+    <tableColumn id="1" xr3:uid="{4976F6FD-69E7-46E4-B49F-470CB1054B48}" name="${module}" dataDxfId="20"/>
+    <tableColumn id="2" xr3:uid="{F5245C18-BA71-4C91-88F9-FA238A6A2D4D}" name="${dataset_id}" dataDxfId="19"/>
+    <tableColumn id="3" xr3:uid="{4046FD08-D747-4231-82F5-17A600D3E724}" name="${username}" dataDxfId="18"/>
+    <tableColumn id="4" xr3:uid="{FBEEF32A-E8E8-4E6F-A05E-10E6A4689538}" name="${password}" dataDxfId="17"/>
+    <tableColumn id="5" xr3:uid="{BBBF3383-D2A3-443A-B066-35CEBE6A0DCF}" name="${role}" dataDxfId="16"/>
+    <tableColumn id="6" xr3:uid="{FFF3448B-D728-4BFB-8F56-81A8FC0AC0DC}" name="${tipo}" dataDxfId="15"/>
+    <tableColumn id="7" xr3:uid="{627C75CC-31B9-4230-8E9A-6B2A4F1A3E6F}" name="${expected_result}" dataDxfId="14"/>
+    <tableColumn id="8" xr3:uid="{DA869EDF-F801-447F-AB76-1E28982A4E9D}" name="${RF}" dataDxfId="13"/>
+    <tableColumn id="9" xr3:uid="{40726AA5-C158-4170-AF35-03DBF46E59E6}" name="${accion}" dataDxfId="12"/>
+    <tableColumn id="10" xr3:uid="{F473F2A5-D7E5-40FF-80EF-B18B0504175C}" name="${campo_url_login}" dataDxfId="11"/>
+    <tableColumn id="11" xr3:uid="{E4A9ED2B-154A-4E07-A3D3-3E8B0EB7662A}" name="${campo_url_target}" dataDxfId="10"/>
+    <tableColumn id="12" xr3:uid="{74E8A3EF-3F1F-4E69-82DE-3C0D9FF3BFF1}" name="${campo_user_locator}" dataDxfId="9"/>
+    <tableColumn id="13" xr3:uid="{FDE67EA9-2B9C-46D5-9C05-283FC050BB68}" name="${campo_pass_locator}" dataDxfId="8"/>
+    <tableColumn id="14" xr3:uid="{3F4A6565-B175-4200-8CD1-D2AA0122ABD9}" name="${campo_submit_locator}" dataDxfId="7"/>
+    <tableColumn id="15" xr3:uid="{2AF443CA-A5EA-401B-9777-981D622C02EF}" name="${campo_dashboard_locator}" dataDxfId="6"/>
+    <tableColumn id="16" xr3:uid="{83424C47-D770-4BE9-8442-5725F667ECD1}" name="${campo_logout_locator}" dataDxfId="5"/>
+    <tableColumn id="17" xr3:uid="{7EEE2949-909D-410F-952D-B9F1D152C5AD}" name="${campo_error_locator}" dataDxfId="4"/>
+    <tableColumn id="18" xr3:uid="{1F68B334-E4E9-4EEE-A3E4-188E3AFD24EA}" name="${expected_error_text}" dataDxfId="3"/>
+    <tableColumn id="19" xr3:uid="{6956A1B5-B972-4BEB-80EF-AE0E78A64242}" name="${campo_bloqueo_locator}" dataDxfId="2"/>
+    <tableColumn id="20" xr3:uid="{F4C1388D-5BD9-4F61-8FCF-C13B6D0FB785}" name="${expected_bloqueo_text}" dataDxfId="1"/>
+    <tableColumn id="21" xr3:uid="{6B400DAD-0A5C-45C1-AE39-96C60BBDC24C}" name="${estado_bug}" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{02D5C7BE-8119-42FD-B7C9-9F8DDD0F56A2}" name="Tabla6" displayName="Tabla6" ref="A1:AE4" totalsRowShown="0" headerRowDxfId="32" dataDxfId="31">
-  <autoFilter ref="A1:AE4" xr:uid="{02D5C7BE-8119-42FD-B7C9-9F8DDD0F56A2}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{02D5C7BE-8119-42FD-B7C9-9F8DDD0F56A2}" name="Tabla6" displayName="Tabla6" ref="A1:AE5" totalsRowShown="0" headerRowDxfId="144" dataDxfId="143">
+  <autoFilter ref="A1:AE5" xr:uid="{02D5C7BE-8119-42FD-B7C9-9F8DDD0F56A2}"/>
   <tableColumns count="31">
-    <tableColumn id="31" xr3:uid="{CE860740-56C7-4E74-BD87-A9479D23FB67}" name="* Test Cases*" dataDxfId="30"/>
-    <tableColumn id="1" xr3:uid="{70447005-0896-47E6-B102-94D445724257}" name="${module}" dataDxfId="29"/>
-    <tableColumn id="2" xr3:uid="{DF799F00-0E1B-4DE8-A033-1CF3F24C51F4}" name="${dataset_id}" dataDxfId="28"/>
-    <tableColumn id="3" xr3:uid="{E153A697-9223-4F5E-97DD-F50968C7F6CF}" name="${pet_id}" dataDxfId="27"/>
-    <tableColumn id="4" xr3:uid="{58D2B8E1-3A26-453B-9353-D23AF2D85023}" name="${nombre}" dataDxfId="26"/>
-    <tableColumn id="5" xr3:uid="{42CC03C9-8646-4C0D-AB7C-0DA19F0993B9}" name="${raza}" dataDxfId="25"/>
-    <tableColumn id="6" xr3:uid="{0262FE2B-D70F-4F83-BF3F-7323B11308C0}" name="${edad}" dataDxfId="24"/>
-    <tableColumn id="7" xr3:uid="{F112F0DD-E45D-4EB9-B1D0-AD91180944AE}" name="${peso}" dataDxfId="23"/>
-    <tableColumn id="8" xr3:uid="{8BCD5B48-E3C8-4085-A53D-BE223385036A}" name="${medicamento_id}" dataDxfId="22"/>
-    <tableColumn id="9" xr3:uid="{1D112CF8-666F-4A83-842D-D3681A10ECEE}" name="${cliente_id}" dataDxfId="21"/>
-    <tableColumn id="10" xr3:uid="{A30B0E0E-5899-4FE0-A2BE-43BB2A3F2311}" name="${tipo}" dataDxfId="20"/>
-    <tableColumn id="11" xr3:uid="{25C19521-DDEE-4788-9B65-2622CA01E93E}" name="${expected_result}" dataDxfId="19"/>
-    <tableColumn id="12" xr3:uid="{FF808F9C-5868-44D7-8884-8C86DB45A951}" name="${RF}" dataDxfId="18"/>
-    <tableColumn id="13" xr3:uid="{DB5E4A5B-0139-4479-837C-685694A14BFF}" name="${accion}" dataDxfId="17"/>
-    <tableColumn id="14" xr3:uid="{C48EE594-3D48-48A3-ADA2-3792C0BE65C1}" name="${nota_defecto}" dataDxfId="16"/>
-    <tableColumn id="15" xr3:uid="{1A61AC86-FF29-48AC-BE01-8F9D46B18BCE}" name="${estado_bug}" dataDxfId="15"/>
-    <tableColumn id="16" xr3:uid="{1455A2D1-0AAB-4769-94A8-54B1129ABFF4}" name="${campo_id_locator}" dataDxfId="14"/>
-    <tableColumn id="17" xr3:uid="{18EFE5B6-918D-4490-B55F-190788A4A0FB}" name="${campo_nombre_locator}" dataDxfId="13"/>
-    <tableColumn id="18" xr3:uid="{D50F63A9-6BC0-4FAD-BC62-AB14ACA1D066}" name="${campo_raza_locator}" dataDxfId="12"/>
-    <tableColumn id="19" xr3:uid="{7E1FDD37-29C3-4206-A1B5-C7BA2B0AE21F}" name="${campo_edad_locator}" dataDxfId="11"/>
-    <tableColumn id="20" xr3:uid="{56866A3F-C743-4485-BB77-92328BDE9A10}" name="${campo_peso_locator}" dataDxfId="10"/>
-    <tableColumn id="21" xr3:uid="{E4D59961-DE22-441D-A07F-C2D61346AD20}" name="${campo_medicamento_locator}" dataDxfId="9"/>
-    <tableColumn id="22" xr3:uid="{AA7ACE5F-D4E1-4224-A784-CD76EDA1B1B8}" name="${campo_cliente_locator}" dataDxfId="8"/>
-    <tableColumn id="23" xr3:uid="{BD6E8966-0C98-4E9B-8748-F820D0ABEB62}" name="${campo_submit_locator}" dataDxfId="7"/>
-    <tableColumn id="24" xr3:uid="{F1B8919B-1DBA-47D6-BFE1-49F1F988A5B7}" name="${campo_edit_btn_locator}" dataDxfId="6"/>
-    <tableColumn id="25" xr3:uid="{C5625C6E-B7E5-411C-84F2-2D4D80F23501}" name="${campo_del_btn_locator}" dataDxfId="5"/>
-    <tableColumn id="26" xr3:uid="{042D884A-20A3-43AD-9757-0A89BC1CD60F}" name="${campo_confirm_del_locator}" dataDxfId="4"/>
-    <tableColumn id="27" xr3:uid="{037CD341-EF51-41FD-8BC8-673E17C1881E}" name="${campo_listado_locator}" dataDxfId="3"/>
-    <tableColumn id="28" xr3:uid="{46737215-83E1-4861-8B08-535057071A1E}" name="${campo_row_search_text}" dataDxfId="2"/>
-    <tableColumn id="29" xr3:uid="{19391385-34B9-449F-B79A-47C49243F480}" name="${username}" dataDxfId="1"/>
-    <tableColumn id="30" xr3:uid="{CE66C601-0577-4B1B-96B0-9CA9147997E9}" name="${password}" dataDxfId="0"/>
+    <tableColumn id="31" xr3:uid="{CE860740-56C7-4E74-BD87-A9479D23FB67}" name="* Test Cases*" dataDxfId="142"/>
+    <tableColumn id="1" xr3:uid="{70447005-0896-47E6-B102-94D445724257}" name="${module}" dataDxfId="141"/>
+    <tableColumn id="2" xr3:uid="{DF799F00-0E1B-4DE8-A033-1CF3F24C51F4}" name="${dataset_id}" dataDxfId="140"/>
+    <tableColumn id="3" xr3:uid="{E153A697-9223-4F5E-97DD-F50968C7F6CF}" name="${pet_id}" dataDxfId="139"/>
+    <tableColumn id="4" xr3:uid="{58D2B8E1-3A26-453B-9353-D23AF2D85023}" name="${nombre}" dataDxfId="138"/>
+    <tableColumn id="5" xr3:uid="{42CC03C9-8646-4C0D-AB7C-0DA19F0993B9}" name="${raza}" dataDxfId="137"/>
+    <tableColumn id="6" xr3:uid="{0262FE2B-D70F-4F83-BF3F-7323B11308C0}" name="${edad}" dataDxfId="136"/>
+    <tableColumn id="7" xr3:uid="{F112F0DD-E45D-4EB9-B1D0-AD91180944AE}" name="${peso}" dataDxfId="135"/>
+    <tableColumn id="8" xr3:uid="{8BCD5B48-E3C8-4085-A53D-BE223385036A}" name="${medicamento_id}" dataDxfId="134"/>
+    <tableColumn id="9" xr3:uid="{1D112CF8-666F-4A83-842D-D3681A10ECEE}" name="${cliente_id}" dataDxfId="133"/>
+    <tableColumn id="10" xr3:uid="{A30B0E0E-5899-4FE0-A2BE-43BB2A3F2311}" name="${tipo}" dataDxfId="132"/>
+    <tableColumn id="11" xr3:uid="{25C19521-DDEE-4788-9B65-2622CA01E93E}" name="${expected_result}" dataDxfId="131"/>
+    <tableColumn id="12" xr3:uid="{FF808F9C-5868-44D7-8884-8C86DB45A951}" name="${RF}" dataDxfId="130"/>
+    <tableColumn id="13" xr3:uid="{DB5E4A5B-0139-4479-837C-685694A14BFF}" name="${accion}" dataDxfId="129"/>
+    <tableColumn id="14" xr3:uid="{C48EE594-3D48-48A3-ADA2-3792C0BE65C1}" name="${nota_defecto}" dataDxfId="128"/>
+    <tableColumn id="15" xr3:uid="{1A61AC86-FF29-48AC-BE01-8F9D46B18BCE}" name="${estado_bug}" dataDxfId="127"/>
+    <tableColumn id="16" xr3:uid="{1455A2D1-0AAB-4769-94A8-54B1129ABFF4}" name="${campo_id_locator}" dataDxfId="126"/>
+    <tableColumn id="17" xr3:uid="{18EFE5B6-918D-4490-B55F-190788A4A0FB}" name="${campo_nombre_locator}" dataDxfId="125"/>
+    <tableColumn id="18" xr3:uid="{D50F63A9-6BC0-4FAD-BC62-AB14ACA1D066}" name="${campo_raza_locator}" dataDxfId="124"/>
+    <tableColumn id="19" xr3:uid="{7E1FDD37-29C3-4206-A1B5-C7BA2B0AE21F}" name="${campo_edad_locator}" dataDxfId="123"/>
+    <tableColumn id="20" xr3:uid="{56866A3F-C743-4485-BB77-92328BDE9A10}" name="${campo_peso_locator}" dataDxfId="122"/>
+    <tableColumn id="21" xr3:uid="{E4D59961-DE22-441D-A07F-C2D61346AD20}" name="${campo_medicamento_locator}" dataDxfId="121"/>
+    <tableColumn id="22" xr3:uid="{AA7ACE5F-D4E1-4224-A784-CD76EDA1B1B8}" name="${campo_cliente_locator}" dataDxfId="120"/>
+    <tableColumn id="23" xr3:uid="{BD6E8966-0C98-4E9B-8748-F820D0ABEB62}" name="${campo_submit_locator}" dataDxfId="119"/>
+    <tableColumn id="24" xr3:uid="{F1B8919B-1DBA-47D6-BFE1-49F1F988A5B7}" name="${campo_edit_btn_locator}" dataDxfId="118"/>
+    <tableColumn id="25" xr3:uid="{C5625C6E-B7E5-411C-84F2-2D4D80F23501}" name="${campo_del_btn_locator}" dataDxfId="117"/>
+    <tableColumn id="26" xr3:uid="{042D884A-20A3-43AD-9757-0A89BC1CD60F}" name="${campo_confirm_del_locator}" dataDxfId="116"/>
+    <tableColumn id="27" xr3:uid="{037CD341-EF51-41FD-8BC8-673E17C1881E}" name="${campo_listado_locator}" dataDxfId="115"/>
+    <tableColumn id="28" xr3:uid="{46737215-83E1-4861-8B08-535057071A1E}" name="${campo_row_search_text}" dataDxfId="114"/>
+    <tableColumn id="29" xr3:uid="{19391385-34B9-449F-B79A-47C49243F480}" name="${username}" dataDxfId="113"/>
+    <tableColumn id="30" xr3:uid="{CE66C601-0577-4B1B-96B0-9CA9147997E9}" name="${password}" dataDxfId="112"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2790,7 +2808,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:AE4"/>
+  <dimension ref="A1:AE5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -3176,6 +3194,95 @@
         <v>88</v>
       </c>
     </row>
+    <row r="5" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="B5" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="M5" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="N5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="O5" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="P5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="Q5" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="R5" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="S5" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="T5" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="U5" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="V5" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="W5" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="X5" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="Z5" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="AA5" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="AB5" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="AC5" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="AD5" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="AE5" s="1" t="s">
+        <v>88</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>